<commit_message>
RAIS+ output is generated
</commit_message>
<xml_diff>
--- a/docs/RAIS - Assistance.xlsx
+++ b/docs/RAIS - Assistance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\amice13\GIT\idp-validator-ua\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70DCED6A-406D-47D3-8698-6C11ADB4C73E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB9CA1DD-B7DD-4548-B4F3-C3212807B996}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{B91F5D51-8A13-488D-B3D2-0AEE8D5D4653}"/>
   </bookViews>
@@ -510,9 +510,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -947,11 +949,12 @@
   <dimension ref="A1:AB2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="28" width="24.47265625" customWidth="1"/>
+    <col min="1" max="1" width="24.47265625" style="3" customWidth="1"/>
+    <col min="2" max="28" width="24.47265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1037,7 +1040,7 @@
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B2" t="s">
@@ -1128,99 +1131,6 @@
       <formula>NOT(ISERROR(FIND("*",A1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="10">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T1:V1 J1:L1" xr:uid="{28E180D2-0016-4760-BEAB-9084D75EC070}">
-      <formula1>AND(
-      SUMPRODUCT(
-        --ISNUMBER(
-          FIND(
-            MID(
-              J1,
-              ROW(INDIRECT("1:"&amp;LEN(J1))),
-              1
-            ),
-            "АБВГҐДЕЄЖЗИІЇЙКЛМНОПРСТУФХЦЧШЩЬЮЯабвгґдеєжзиіїйклмнопрстуфхцчшщьюя-'IVXCLD0123456789."
-          )
-        )
-      )=LEN(J1),
-      LEN(J1) &lt;= 5
-    )</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I1 S1" xr:uid="{C7CD8BF0-F3D8-448A-AE54-EE330D57A28D}">
-      <formula1>SUMPRODUCT(
-      --ISNUMBER(
-        FIND(
-          MID(
-            I1,
-            ROW(INDIRECT("1:"&amp;LEN(I1))),
-            1
-          ),
-          "АБВГҐДЕЄЖЗИІЇЙКЛМНОПРСТУФХЦЧШЩЬЮЯабвгґдеєжзиіїйклмнопрстуфхцчшщьюя-'IVXCLD0123456789. "
-        )
-      )
-    )=LEN(I1)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H1 R1" xr:uid="{1107B492-A8D3-4739-AC9C-0C58139FFCF1}">
-      <formula1>INDIRECT("StreetTypes[Street Type]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G1 Q1" xr:uid="{357FEDCE-A87E-4875-81A9-C8E550ADA13A}">
-      <formula1>OFFSET(
-      INDEX(INDIRECT("Admin4[Admin 4 Parent]"),1),
-      MATCH(
-        LEFT(RIGHT(F1,10),9),
-        INDIRECT("Admin4[Admin 4 Parent]"),
-      0) - 1,
-      1,
-      COUNTIF(
-        INDIRECT("Admin4[Admin 4 Parent]"),
-        LEFT(RIGHT(F1,10),9)
-      ),
-      1
-    )</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F1 P1" xr:uid="{B3223EC3-55BD-4516-A3FE-9A056E494542}">
-      <formula1>OFFSET(
-      INDEX(INDIRECT("Admin3[Admin 3 Parent]"),1),
-      MATCH(
-        LEFT(RIGHT(E1,7),6),
-        INDIRECT("Admin3[Admin 3 Parent]"),
-      0) - 1,
-      1,
-      COUNTIF(
-        INDIRECT("Admin3[Admin 3 Parent]"),
-        LEFT(RIGHT(E1,7),6)
-      ),
-      1
-    )</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1 O1" xr:uid="{2D92D83B-2873-42CA-8071-72E47010BD7A}">
-      <formula1>OFFSET(
-      INDEX(INDIRECT("Admin2[Admin 2 Parent]"),1),
-      MATCH(
-        LEFT(RIGHT(D1,5),4),
-        INDIRECT("Admin2[Admin 2 Parent]"),
-      0) - 1,
-      1,
-      COUNTIF(
-        INDIRECT("Admin2[Admin 2 Parent]"),
-        LEFT(RIGHT(D1,5),4)
-      ),
-      1
-    )</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1 N1" xr:uid="{16E932D1-7292-48B1-8CA9-183834276E83}">
-      <formula1>INDIRECT("Admin1[Admin 1 Name]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1 M1" xr:uid="{0B5EDD30-A92F-4DDC-8E51-07724DE4E9D1}">
-      <formula1>INDIRECT("Countries[Country Name]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1" xr:uid="{CBBE4451-39FD-4E28-96D3-3A0FA0731861}">
-      <formula1>INDIRECT("PopulationTypes[Population Type]")</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A1 W1:Z1" xr:uid="{5BC970B4-934B-478F-A440-F085606F3AE5}">
-      <formula1>INDIRECT("Households[Household]")</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>